<commit_message>
Restore the PR #7 work removed by the revert in PR #13
PR #13 («Revert "Pop"») undid PR #12, and with it the merged PR #7 and #6 work:
model/wac.py, model/monthly_standard.py, model/tests/, the monthly/ intake folders,
the casing and single-material recipes in costing_pricing_model.py, and their
reports. This puts the repository back to the tree of 87d4b19 (the PR #7 merge),
file for file. Nothing newer than that tree was on main.

The six files uploaded in 73def48 (the 2025 income statement text and
«قائمة دخل تفصيلى .xlsx»), also removed by the revert, are not restored here.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JRoSvdJwzkvyrFQxPzaBvo
</commit_message>
<xml_diff>
--- a/ABOHASHEM_Costing_Pricing_Model_June2026.xlsx
+++ b/ABOHASHEM_Costing_Pricing_Model_June2026.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="١. الملخص التنفيذي" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="٢. تقرير جودة البيانات" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="٣. التكلفة المعيارية" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="٤. التكلفة الفعلية والانحرافات" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="٥. توزيع المصروفات" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="٦. تحليل الربحية" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="٧. تحليل المبيعات ABC" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="٨. قائمة الأسعار المقترحة" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="٩. قواعد التسعير والتنبيهات" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="١٠. المنهجية والافتراضات" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="١١. الإعدادات" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="١. الملخص التنفيذي" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="٢. تقرير جودة البيانات" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="٣. التكلفة المعيارية" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="٤. التكلفة الفعلية والانحرافات" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="٥. توزيع المصروفات" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="٦. تحليل الربحية" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="٧. تحليل المبيعات ABC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="٨. قائمة الأسعار المقترحة" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="٩. قواعد التسعير والتنبيهات" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="١٠. المنهجية والافتراضات" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="١١. الإعدادات" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
@@ -943,10 +943,10 @@
         <v>0.4298787741909529</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>0.5056860757820014</v>
+        <v>0.4865287808065942</v>
       </c>
       <c r="E19" s="11" t="n">
-        <v>0.1203138823222033</v>
+        <v>0.1094685334336097</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>12</v>
@@ -959,16 +959,16 @@
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>955422.9901890159</v>
+        <v>955422.9901890161</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>0.2553397134269581</v>
+        <v>0.2553397134269582</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.490409049286595</v>
+        <v>0.5197451980295722</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>0.1156070071938775</v>
+        <v>0.1322148199656547</v>
       </c>
       <c r="F20" s="9" t="n">
         <v>8</v>
@@ -981,16 +981,16 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>907477.5075514012</v>
+        <v>907477.5075514013</v>
       </c>
       <c r="C21" s="11" t="n">
         <v>0.2425261366944328</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>0.2850093903283707</v>
+        <v>0.2396477491593181</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>0.07165101552548038</v>
+        <v>0.04597083336671956</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>10</v>
@@ -1009,10 +1009,10 @@
         <v>0.07225537568765614</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.7589860578707998</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>0.1843474543310752</v>
+        <v>0.2763775135120883</v>
       </c>
       <c r="F22" s="9" t="n">
         <v>3</v>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>10 أصناف تجارية بلا تركيبة خامات: بانيه 800 جرام، بانيه 900 جرام اسباشيل، استربس الهنا 800 جرام، عجينة بقري 5 ك، مفروم صافي 400 جم (ابو هاشم)، استريس اسبشيال 900 جرام… — احتُسبت تكلفتها الفعلية بالتناسب مع تكلفة المبيعات (غير معيارية).</t>
+          <t>7 أصناف تجارية بلا تركيبة خامات: بانيه 800 جرام، بانيه 900 جرام اسباشيل، استربس الهنا 800 جرام، عجينة بقري 5 ك، استريس اسبشيال 900 جرام، استربس الهنا 900 جرام… — احتُسبت تكلفتها الفعلية بالتناسب مع تكلفة المبيعات (غير معيارية).</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>2 أصناف بهامش تشغيلي سالب: كفته الهنا 350، عجينه سجق 5 كيلو الهنا — تبيع دون التكلفة المحمّلة.</t>
+          <t>4 أصناف بهامش تشغيلي سالب: كفته الهنا 350، مفروم صافي 400 جم (ابو هاشم)، عجينه سجق 5 كيلو الهنا، كيلو مفروم هندي — تبيع دون التكلفة المحمّلة.</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>2 صنف سعره الحالي &lt; التكلفة المحمّلة بالكامل — مدرجة في محرك التسعير للرفع.</t>
+          <t>3 صنف سعره الحالي &lt; التكلفة المحمّلة بالكامل — مدرجة في محرك التسعير للرفع.</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
         <v>3</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>273.2502</v>
+        <v>262.7192</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>9.23</v>
@@ -1772,13 +1772,13 @@
         <v>0.2687</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>2.8248</v>
+        <v>2.7195</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>1.4124</v>
+        <v>1.3597</v>
       </c>
       <c r="M4" s="17" t="n">
-        <v>321.3131</v>
+        <v>310.6241</v>
       </c>
     </row>
     <row r="5">
@@ -1979,7 +1979,7 @@
         <v>0.8</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>22.254</v>
+        <v>11.884</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>0</v>
@@ -1997,13 +1997,13 @@
         <v>0.0717</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>0.2225</v>
+        <v>0.1188</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>0.1113</v>
+        <v>0.0594</v>
       </c>
       <c r="M9" s="18" t="n">
-        <v>31.8134</v>
+        <v>21.2878</v>
       </c>
     </row>
     <row r="10">
@@ -2069,7 +2069,7 @@
         <v>0.9</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>24.2393</v>
+        <v>12.9442</v>
       </c>
       <c r="F11" s="8" t="n">
         <v>0</v>
@@ -2087,13 +2087,13 @@
         <v>0.0806</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>0.2424</v>
+        <v>0.1294</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>0.1212</v>
+        <v>0.06469999999999999</v>
       </c>
       <c r="M11" s="18" t="n">
-        <v>34.9816</v>
+        <v>23.5171</v>
       </c>
     </row>
     <row r="12">
@@ -2114,7 +2114,7 @@
         <v>0.8</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>58.506</v>
+        <v>31.2432</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0</v>
@@ -2132,13 +2132,13 @@
         <v>0.0717</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>0.5851</v>
+        <v>0.3124</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>0.2925</v>
+        <v>0.1562</v>
       </c>
       <c r="M12" s="17" t="n">
-        <v>68.6091</v>
+        <v>40.9373</v>
       </c>
     </row>
     <row r="13">
@@ -2204,7 +2204,7 @@
         <v>5</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>119.0305</v>
+        <v>202.3638</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>16.06</v>
@@ -2222,13 +2222,13 @@
         <v>0.4478</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>1.3509</v>
+        <v>2.1842</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>0.6755</v>
+        <v>1.0921</v>
       </c>
       <c r="M14" s="17" t="n">
-        <v>194.7764</v>
+        <v>279.3597</v>
       </c>
     </row>
     <row r="15">
@@ -2249,7 +2249,7 @@
         <v>0.35</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>8.332100000000001</v>
+        <v>13.3321</v>
       </c>
       <c r="F15" s="8" t="n">
         <v>4.63</v>
@@ -2267,13 +2267,13 @@
         <v>0.0313</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>0.1296</v>
+        <v>0.1796</v>
       </c>
       <c r="L15" s="8" t="n">
-        <v>0.0648</v>
+        <v>0.0898</v>
       </c>
       <c r="M15" s="18" t="n">
-        <v>17.1927</v>
+        <v>22.2677</v>
       </c>
     </row>
     <row r="16">
@@ -2384,7 +2384,7 @@
         <v>5</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>178.4109</v>
+        <v>95.2743</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>0</v>
@@ -2402,13 +2402,13 @@
         <v>0.4478</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>1.7841</v>
+        <v>0.9527</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>0.8921</v>
+        <v>0.4764</v>
       </c>
       <c r="M18" s="17" t="n">
-        <v>238.7465</v>
+        <v>154.363</v>
       </c>
     </row>
     <row r="19">
@@ -2429,10 +2429,10 @@
         <v>0.4</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>37.665</v>
+        <v>80.95999999999999</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="G19" s="8" t="n">
         <v>0.8255</v>
@@ -2447,13 +2447,13 @@
         <v>0.0358</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>0.3766</v>
+        <v>0.8721</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>0.1883</v>
+        <v>0.4361</v>
       </c>
       <c r="M19" s="18" t="n">
-        <v>42.8427</v>
+        <v>93.1309</v>
       </c>
     </row>
     <row r="20">
@@ -2474,7 +2474,7 @@
         <v>0.9</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>64.2689</v>
+        <v>34.3206</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0</v>
@@ -2492,13 +2492,13 @@
         <v>0.0806</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>0.6427</v>
+        <v>0.3432</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>0.3213</v>
+        <v>0.1716</v>
       </c>
       <c r="M20" s="17" t="n">
-        <v>75.6116</v>
+        <v>45.2142</v>
       </c>
     </row>
     <row r="21">
@@ -2519,10 +2519,10 @@
         <v>0.4</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>29.6909</v>
+        <v>57.6267</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="G21" s="8" t="n">
         <v>0.8255</v>
@@ -2537,13 +2537,13 @@
         <v>0.0358</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>0.2969</v>
+        <v>0.6388</v>
       </c>
       <c r="L21" s="8" t="n">
-        <v>0.1485</v>
+        <v>0.3194</v>
       </c>
       <c r="M21" s="18" t="n">
-        <v>34.7491</v>
+        <v>69.44759999999999</v>
       </c>
     </row>
     <row r="22">
@@ -2609,7 +2609,7 @@
         <v>0.8</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>19.0449</v>
+        <v>30.7115</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>5.99</v>
@@ -2627,13 +2627,13 @@
         <v>0.0717</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>0.2503</v>
+        <v>0.367</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>0.1252</v>
+        <v>0.1835</v>
       </c>
       <c r="M23" s="18" t="n">
-        <v>34.6359</v>
+        <v>46.4776</v>
       </c>
     </row>
     <row r="24">
@@ -2699,7 +2699,7 @@
         <v>0.8</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>72.86669999999999</v>
+        <v>70.0585</v>
       </c>
       <c r="F25" s="8" t="n">
         <v>6.27</v>
@@ -2717,13 +2717,13 @@
         <v>0.0717</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>0.7914</v>
+        <v>0.7633</v>
       </c>
       <c r="L25" s="8" t="n">
-        <v>0.3957</v>
+        <v>0.3816</v>
       </c>
       <c r="M25" s="18" t="n">
-        <v>89.5493</v>
+        <v>86.69889999999999</v>
       </c>
     </row>
     <row r="26">
@@ -2744,7 +2744,7 @@
         <v>0.3</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>8.333299999999999</v>
+        <v>13.3333</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>5.2</v>
@@ -2762,13 +2762,13 @@
         <v>0.0269</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>0.1353</v>
+        <v>0.1853</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>0.0677</v>
+        <v>0.0927</v>
       </c>
       <c r="M26" s="17" t="n">
-        <v>17.1959</v>
+        <v>22.2709</v>
       </c>
     </row>
     <row r="27">
@@ -2789,7 +2789,7 @@
         <v>0.7</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>19.4445</v>
+        <v>31.1111</v>
       </c>
       <c r="F27" s="8" t="n">
         <v>7.2</v>
@@ -2807,13 +2807,13 @@
         <v>0.06270000000000001</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>0.2664</v>
+        <v>0.3831</v>
       </c>
       <c r="L27" s="8" t="n">
-        <v>0.1332</v>
+        <v>0.1916</v>
       </c>
       <c r="M27" s="18" t="n">
-        <v>35.1165</v>
+        <v>46.9581</v>
       </c>
     </row>
     <row r="28">
@@ -3014,7 +3014,7 @@
         <v>0.35</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>31.8792</v>
+        <v>30.6506</v>
       </c>
       <c r="F32" s="5" t="n">
         <v>4.67</v>
@@ -3032,13 +3032,13 @@
         <v>0.0313</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>0.3655</v>
+        <v>0.3532</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>0.1827</v>
+        <v>0.1766</v>
       </c>
       <c r="M32" s="17" t="n">
-        <v>41.1336</v>
+        <v>39.8865</v>
       </c>
     </row>
     <row r="33">
@@ -3059,10 +3059,10 @@
         <v>1</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>103.3411</v>
+        <v>253</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>2.0637</v>
@@ -3077,13 +3077,13 @@
         <v>0.0896</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>1.0334</v>
+        <v>2.55</v>
       </c>
       <c r="L33" s="8" t="n">
-        <v>0.5167</v>
+        <v>1.275</v>
       </c>
       <c r="M33" s="18" t="n">
-        <v>116.4231</v>
+        <v>270.3569</v>
       </c>
     </row>
     <row r="34">
@@ -3149,7 +3149,7 @@
         <v>0.9</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>60.5209</v>
+        <v>32.3192</v>
       </c>
       <c r="F35" s="8" t="n">
         <v>0</v>
@@ -3167,13 +3167,13 @@
         <v>0.0806</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>0.6052</v>
+        <v>0.3232</v>
       </c>
       <c r="L35" s="8" t="n">
-        <v>0.3026</v>
+        <v>0.1616</v>
       </c>
       <c r="M35" s="18" t="n">
-        <v>71.8074</v>
+        <v>43.1827</v>
       </c>
     </row>
     <row r="36">
@@ -3194,7 +3194,7 @@
         <v>1</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>46.8549</v>
+        <v>25.0213</v>
       </c>
       <c r="F36" s="5" t="n">
         <v>0</v>
@@ -3212,13 +3212,13 @@
         <v>0.0896</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>0.4685</v>
+        <v>0.2502</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>0.2343</v>
+        <v>0.1251</v>
       </c>
       <c r="M36" s="17" t="n">
-        <v>59.0896</v>
+        <v>36.9285</v>
       </c>
     </row>
     <row r="37" ht="40" customHeight="1">
@@ -3344,10 +3344,10 @@
         <v>1607</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>321.313</v>
+        <v>310.624</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>317.076</v>
+        <v>306.545</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>0</v>
@@ -3359,7 +3359,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-6809.185</v>
+        <v>-6555.335</v>
       </c>
       <c r="J4" s="11" t="n">
         <v>1.013</v>
@@ -3539,10 +3539,10 @@
         <v>3412</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>31.813</v>
+        <v>21.288</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>31.48</v>
+        <v>21.11</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>0</v>
@@ -3554,10 +3554,10 @@
         <v>0</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>-1138.961</v>
+        <v>-608.224</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>1.011</v>
+        <v>1.008</v>
       </c>
       <c r="K9" s="20" t="inlineStr">
         <is>
@@ -3617,10 +3617,10 @@
         <v>2500</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>34.982</v>
+        <v>23.517</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>34.618</v>
+        <v>23.323</v>
       </c>
       <c r="F11" s="8" t="n">
         <v>0</v>
@@ -3632,10 +3632,10 @@
         <v>-0</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>-908.973</v>
+        <v>-485.407</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.011</v>
+        <v>1.008</v>
       </c>
       <c r="K11" s="20" t="inlineStr">
         <is>
@@ -3656,10 +3656,10 @@
         <v>935</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>68.60899999999999</v>
+        <v>40.937</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>67.732</v>
+        <v>40.469</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0</v>
@@ -3671,10 +3671,10 @@
         <v>-0</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-820.547</v>
+        <v>-438.185</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>1.013</v>
+        <v>1.012</v>
       </c>
       <c r="K12" s="20" t="inlineStr">
         <is>
@@ -3734,10 +3734,10 @@
         <v>358</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>194.776</v>
+        <v>279.36</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>192.75</v>
+        <v>276.083</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>0</v>
@@ -3749,10 +3749,10 @@
         <v>-0</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-725.436</v>
+        <v>-1172.936</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>1.011</v>
+        <v>1.012</v>
       </c>
       <c r="K14" s="20" t="inlineStr">
         <is>
@@ -3773,10 +3773,10 @@
         <v>3375</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>17.193</v>
+        <v>22.268</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>16.998</v>
+        <v>21.998</v>
       </c>
       <c r="F15" s="8" t="n">
         <v>0</v>
@@ -3788,10 +3788,10 @@
         <v>-0</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>-656.208</v>
+        <v>-909.333</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>1.011</v>
+        <v>1.012</v>
       </c>
       <c r="K15" s="20" t="inlineStr">
         <is>
@@ -3890,10 +3890,10 @@
         <v>166</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>238.747</v>
+        <v>154.363</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>236.07</v>
+        <v>152.934</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>0</v>
@@ -3905,10 +3905,10 @@
         <v>0</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>-444.243</v>
+        <v>-237.233</v>
       </c>
       <c r="J18" s="11" t="n">
-        <v>1.011</v>
+        <v>1.009</v>
       </c>
       <c r="K18" s="20" t="inlineStr">
         <is>
@@ -3929,10 +3929,10 @@
         <v>647</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>42.843</v>
+        <v>93.131</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>42.278</v>
+        <v>91.82299999999999</v>
       </c>
       <c r="F19" s="8" t="n">
         <v>0</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>-365.539</v>
+        <v>-846.373</v>
       </c>
       <c r="J19" s="10" t="n">
-        <v>1.013</v>
+        <v>1.014</v>
       </c>
       <c r="K19" s="20" t="inlineStr">
         <is>
@@ -3968,10 +3968,10 @@
         <v>374</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>75.61199999999999</v>
+        <v>45.214</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>74.648</v>
+        <v>44.699</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0</v>
@@ -3983,10 +3983,10 @@
         <v>0</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-360.549</v>
+        <v>-192.539</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>1.013</v>
+        <v>1.012</v>
       </c>
       <c r="K20" s="20" t="inlineStr">
         <is>
@@ -4007,10 +4007,10 @@
         <v>797</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>34.749</v>
+        <v>69.44799999999999</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>34.304</v>
+        <v>68.489</v>
       </c>
       <c r="F21" s="8" t="n">
         <v>0</v>
@@ -4022,10 +4022,10 @@
         <v>0</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>-354.955</v>
+        <v>-763.646</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.013</v>
+        <v>1.014</v>
       </c>
       <c r="K21" s="20" t="inlineStr">
         <is>
@@ -4085,10 +4085,10 @@
         <v>937</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>34.636</v>
+        <v>46.478</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>34.26</v>
+        <v>45.927</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>0</v>
@@ -4100,10 +4100,10 @@
         <v>-0</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>-351.865</v>
+        <v>-515.84</v>
       </c>
       <c r="J23" s="10" t="n">
-        <v>1.011</v>
+        <v>1.012</v>
       </c>
       <c r="K23" s="20" t="inlineStr">
         <is>
@@ -4163,10 +4163,10 @@
         <v>353</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>89.54900000000001</v>
+        <v>86.699</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>88.36199999999999</v>
+        <v>85.554</v>
       </c>
       <c r="F25" s="8" t="n">
         <v>0</v>
@@ -4178,7 +4178,7 @@
         <v>0</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>-419.029</v>
+        <v>-404.159</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>1.013</v>
@@ -4202,10 +4202,10 @@
         <v>1218</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>17.196</v>
+        <v>22.271</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>16.993</v>
+        <v>21.993</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>0</v>
@@ -4217,10 +4217,10 @@
         <v>-0</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>-247.254</v>
+        <v>-338.604</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>1.012</v>
+        <v>1.013</v>
       </c>
       <c r="K26" s="20" t="inlineStr">
         <is>
@@ -4241,10 +4241,10 @@
         <v>456</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>35.116</v>
+        <v>46.958</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>34.717</v>
+        <v>46.383</v>
       </c>
       <c r="F27" s="8" t="n">
         <v>0</v>
@@ -4256,7 +4256,7 @@
         <v>-0</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>-182.248</v>
+        <v>-262.048</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>1.012</v>
@@ -4436,10 +4436,10 @@
         <v>181</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>41.134</v>
+        <v>39.887</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>40.585</v>
+        <v>39.357</v>
       </c>
       <c r="F32" s="5" t="n">
         <v>0</v>
@@ -4451,10 +4451,10 @@
         <v>-0</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>-99.23099999999999</v>
+        <v>-95.895</v>
       </c>
       <c r="J32" s="11" t="n">
-        <v>1.014</v>
+        <v>1.013</v>
       </c>
       <c r="K32" s="20" t="inlineStr">
         <is>
@@ -4475,10 +4475,10 @@
         <v>34.5</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>116.423</v>
+        <v>270.357</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>114.873</v>
+        <v>266.532</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>0</v>
@@ -4490,10 +4490,10 @@
         <v>-0</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>-53.479</v>
+        <v>-131.962</v>
       </c>
       <c r="J33" s="10" t="n">
-        <v>1.013</v>
+        <v>1.014</v>
       </c>
       <c r="K33" s="20" t="inlineStr">
         <is>
@@ -4553,10 +4553,10 @@
         <v>45</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>71.807</v>
+        <v>43.183</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>70.90000000000001</v>
+        <v>42.698</v>
       </c>
       <c r="F35" s="8" t="n">
         <v>0</v>
@@ -4568,10 +4568,10 @@
         <v>-0</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>-40.852</v>
+        <v>-21.815</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>1.013</v>
+        <v>1.011</v>
       </c>
       <c r="K35" s="20" t="inlineStr">
         <is>
@@ -4592,10 +4592,10 @@
         <v>3</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>59.09</v>
+        <v>36.929</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>58.387</v>
+        <v>36.553</v>
       </c>
       <c r="F36" s="5" t="n">
         <v>0</v>
@@ -4607,10 +4607,10 @@
         <v>-0</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>-2.108</v>
+        <v>-1.126</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>1.012</v>
+        <v>1.01</v>
       </c>
       <c r="K36" s="20" t="inlineStr">
         <is>
@@ -5048,19 +5048,19 @@
         </is>
       </c>
       <c r="C31" s="5" t="n">
-        <v>128751.4</v>
+        <v>145674.8</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>0.07565430168215746</v>
+        <v>0.08559843728812898</v>
       </c>
       <c r="E31" s="5" t="n">
         <v>55595.3</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>55862.5</v>
+        <v>63205.2</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>111457.8</v>
+        <v>118800.5</v>
       </c>
     </row>
     <row r="32">
@@ -5173,19 +5173,19 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>112213.9</v>
+        <v>147596.3</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>0.06593682849239532</v>
+        <v>0.08672755774707948</v>
       </c>
       <c r="E36" s="8" t="n">
         <v>31477.5</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>48687.2</v>
+        <v>64038.9</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>80164.7</v>
+        <v>95516.39999999999</v>
       </c>
     </row>
     <row r="37">
@@ -5201,7 +5201,7 @@
         <v>50373.8</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>0.02959965102630487</v>
+        <v>0.02959965102630486</v>
       </c>
       <c r="E37" s="5" t="n">
         <v>34993.6</v>
@@ -5223,19 +5223,19 @@
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>89554.8</v>
+        <v>117792.6</v>
       </c>
       <c r="D38" s="10" t="n">
-        <v>0.05262238081907773</v>
+        <v>0.06921489364326536</v>
       </c>
       <c r="E38" s="8" t="n">
         <v>25946.8</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>38855.9</v>
+        <v>51107.7</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>64802.7</v>
+        <v>77054.5</v>
       </c>
     </row>
     <row r="39">
@@ -5248,19 +5248,19 @@
         </is>
       </c>
       <c r="C39" s="5" t="n">
-        <v>80842.7</v>
+        <v>106333.5</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>0.04750316081877852</v>
+        <v>0.06248151779933683</v>
       </c>
       <c r="E39" s="5" t="n">
         <v>8625.9</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>35076</v>
+        <v>46135.9</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>43701.8</v>
+        <v>54761.7</v>
       </c>
     </row>
     <row r="40">
@@ -5298,19 +5298,19 @@
         </is>
       </c>
       <c r="C41" s="5" t="n">
-        <v>79816</v>
+        <v>49982.6</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>0.04689983848444355</v>
+        <v>0.02936978144864998</v>
       </c>
       <c r="E41" s="5" t="n">
         <v>20642.1</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>34630.5</v>
+        <v>21686.4</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>55272.6</v>
+        <v>42328.5</v>
       </c>
     </row>
     <row r="42">
@@ -5323,19 +5323,19 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>56170.7</v>
+        <v>39295.7</v>
       </c>
       <c r="D42" s="10" t="n">
-        <v>0.03300587356991161</v>
+        <v>0.02309012901754234</v>
       </c>
       <c r="E42" s="8" t="n">
         <v>13622.1</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>24371.3</v>
+        <v>17049.6</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>37993.3</v>
+        <v>30671.6</v>
       </c>
     </row>
     <row r="43">
@@ -5398,19 +5398,19 @@
         </is>
       </c>
       <c r="C45" s="5" t="n">
-        <v>43768.2</v>
+        <v>57568.8</v>
       </c>
       <c r="D45" s="11" t="n">
-        <v>0.02571816379803249</v>
+        <v>0.03382743129964096</v>
       </c>
       <c r="E45" s="5" t="n">
         <v>9571.5</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>18990.1</v>
+        <v>24977.9</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>28561.6</v>
+        <v>34549.4</v>
       </c>
     </row>
     <row r="46">
@@ -5423,19 +5423,19 @@
         </is>
       </c>
       <c r="C46" s="8" t="n">
-        <v>36014</v>
+        <v>3958.3</v>
       </c>
       <c r="D46" s="10" t="n">
-        <v>0.02116179352620703</v>
+        <v>0.002325914067258377</v>
       </c>
       <c r="E46" s="8" t="n">
         <v>2984.5</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>15625.7</v>
+        <v>1717.4</v>
       </c>
       <c r="G46" s="8" t="n">
-        <v>18610.2</v>
+        <v>4701.9</v>
       </c>
     </row>
     <row r="47">
@@ -5448,19 +5448,19 @@
         </is>
       </c>
       <c r="C47" s="5" t="n">
-        <v>35522.3</v>
+        <v>46723</v>
       </c>
       <c r="D47" s="11" t="n">
-        <v>0.02087290920773737</v>
+        <v>0.0274544056797086</v>
       </c>
       <c r="E47" s="5" t="n">
         <v>3881.6</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>15412.4</v>
+        <v>20272.1</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>19294</v>
+        <v>24153.8</v>
       </c>
     </row>
     <row r="48">
@@ -5473,19 +5473,19 @@
         </is>
       </c>
       <c r="C48" s="8" t="n">
-        <v>34971.3</v>
+        <v>7725.2</v>
       </c>
       <c r="D48" s="10" t="n">
-        <v>0.02054910108081422</v>
+        <v>0.004539330273089558</v>
       </c>
       <c r="E48" s="8" t="n">
         <v>3676.4</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>15173.3</v>
+        <v>3351.8</v>
       </c>
       <c r="G48" s="8" t="n">
-        <v>18849.7</v>
+        <v>7028.2</v>
       </c>
     </row>
     <row r="49">
@@ -5501,7 +5501,7 @@
         <v>17741.8</v>
       </c>
       <c r="D49" s="11" t="n">
-        <v>0.01042506017493517</v>
+        <v>0.01042506017493516</v>
       </c>
       <c r="E49" s="5" t="n">
         <v>5466.1</v>
@@ -5523,19 +5523,19 @@
         </is>
       </c>
       <c r="C50" s="8" t="n">
-        <v>32800.9</v>
+        <v>21869.2</v>
       </c>
       <c r="D50" s="10" t="n">
-        <v>0.01927379851919181</v>
+        <v>0.01285035471484711</v>
       </c>
       <c r="E50" s="8" t="n">
         <v>8644.299999999999</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>14231.6</v>
+        <v>9488.6</v>
       </c>
       <c r="G50" s="8" t="n">
-        <v>22875.9</v>
+        <v>18132.9</v>
       </c>
     </row>
     <row r="51">
@@ -5551,7 +5551,7 @@
         <v>12886.9</v>
       </c>
       <c r="D51" s="11" t="n">
-        <v>0.007572334841311312</v>
+        <v>0.007572334841311315</v>
       </c>
       <c r="E51" s="5" t="n">
         <v>4359.1</v>
@@ -5573,19 +5573,19 @@
         </is>
       </c>
       <c r="C52" s="8" t="n">
-        <v>11098.5</v>
+        <v>12089.8</v>
       </c>
       <c r="D52" s="10" t="n">
-        <v>0.006521448283249481</v>
+        <v>0.007103946498376285</v>
       </c>
       <c r="E52" s="8" t="n">
         <v>3256.6</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>4815.4</v>
+        <v>5245.5</v>
       </c>
       <c r="G52" s="8" t="n">
-        <v>8072</v>
+        <v>8502.1</v>
       </c>
     </row>
     <row r="53">
@@ -5598,19 +5598,19 @@
         </is>
       </c>
       <c r="C53" s="5" t="n">
-        <v>21607.1</v>
+        <v>15517.1</v>
       </c>
       <c r="D53" s="11" t="n">
-        <v>0.01269632068310903</v>
+        <v>0.009117838649098433</v>
       </c>
       <c r="E53" s="5" t="n">
         <v>4213.8</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>9374.9</v>
+        <v>6732.5</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>13588.6</v>
+        <v>10946.3</v>
       </c>
     </row>
     <row r="54">
@@ -5623,19 +5623,19 @@
         </is>
       </c>
       <c r="C54" s="8" t="n">
-        <v>19350.2</v>
+        <v>14030.2</v>
       </c>
       <c r="D54" s="10" t="n">
-        <v>0.01137015066112079</v>
+        <v>0.008244120378536814</v>
       </c>
       <c r="E54" s="8" t="n">
         <v>3681</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>8395.6</v>
+        <v>6087.4</v>
       </c>
       <c r="G54" s="8" t="n">
-        <v>12076.6</v>
+        <v>9768.4</v>
       </c>
     </row>
     <row r="55">
@@ -5651,7 +5651,7 @@
         <v>10979.3</v>
       </c>
       <c r="D55" s="11" t="n">
-        <v>0.006451456022974457</v>
+        <v>0.006451456022974458</v>
       </c>
       <c r="E55" s="5" t="n">
         <v>5424.6</v>
@@ -5676,7 +5676,7 @@
         <v>7263.1</v>
       </c>
       <c r="D56" s="10" t="n">
-        <v>0.004267781420178886</v>
+        <v>0.004267781420178885</v>
       </c>
       <c r="E56" s="8" t="n">
         <v>2525.5</v>
@@ -5701,7 +5701,7 @@
         <v>5544</v>
       </c>
       <c r="D57" s="11" t="n">
-        <v>0.003257674799780448</v>
+        <v>0.003257674799780447</v>
       </c>
       <c r="E57" s="5" t="n">
         <v>2232.6</v>
@@ -5748,19 +5748,19 @@
         </is>
       </c>
       <c r="C59" s="5" t="n">
-        <v>2521.1</v>
+        <v>2743.5</v>
       </c>
       <c r="D59" s="11" t="n">
-        <v>0.001481409878290361</v>
+        <v>0.001612080069254536</v>
       </c>
       <c r="E59" s="5" t="n">
         <v>730.5</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>1093.9</v>
+        <v>1190.3</v>
       </c>
       <c r="G59" s="5" t="n">
-        <v>1824.4</v>
+        <v>1920.9</v>
       </c>
     </row>
     <row r="60">
@@ -5773,19 +5773,19 @@
         </is>
       </c>
       <c r="C60" s="8" t="n">
-        <v>5268.9</v>
+        <v>36.7</v>
       </c>
       <c r="D60" s="10" t="n">
-        <v>0.003096012572707114</v>
+        <v>2.155472787556532e-05</v>
       </c>
       <c r="E60" s="8" t="n">
         <v>397.9</v>
       </c>
       <c r="F60" s="8" t="n">
-        <v>2286.1</v>
+        <v>15.9</v>
       </c>
       <c r="G60" s="8" t="n">
-        <v>2683.9</v>
+        <v>413.8</v>
       </c>
     </row>
     <row r="61">
@@ -5801,7 +5801,7 @@
         <v>1847.6</v>
       </c>
       <c r="D61" s="11" t="n">
-        <v>0.00108564633830158</v>
+        <v>0.001085646338301579</v>
       </c>
       <c r="E61" s="5" t="n">
         <v>573.1</v>
@@ -5823,19 +5823,19 @@
         </is>
       </c>
       <c r="C62" s="8" t="n">
-        <v>4024.8</v>
+        <v>5293.9</v>
       </c>
       <c r="D62" s="10" t="n">
-        <v>0.00236498605789422</v>
+        <v>0.003110696549966983</v>
       </c>
       <c r="E62" s="8" t="n">
         <v>467</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>1746.3</v>
+        <v>2296.9</v>
       </c>
       <c r="G62" s="8" t="n">
-        <v>2213.3</v>
+        <v>2764</v>
       </c>
     </row>
     <row r="63">
@@ -5848,19 +5848,19 @@
         </is>
       </c>
       <c r="C63" s="5" t="n">
-        <v>207.7</v>
+        <v>273.2</v>
       </c>
       <c r="D63" s="11" t="n">
-        <v>0.0001220637965364759</v>
+        <v>0.0001605520799982959</v>
       </c>
       <c r="E63" s="5" t="n">
         <v>34.6</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>90.09999999999999</v>
+        <v>118.6</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>124.7</v>
+        <v>153.1</v>
       </c>
     </row>
   </sheetData>
@@ -5984,28 +5984,28 @@
         <v>582697.1</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>565403.5</v>
+        <v>555822.9</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>128751.4</v>
+        <v>145674.8</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>0.2209577350382543</v>
+        <v>0.2500008116585349</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>111457.8</v>
+        <v>118800.5</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>17293.6</v>
+        <v>26874.3</v>
       </c>
       <c r="I4" s="22" t="n">
-        <v>0.02967855287448811</v>
+        <v>0.04612045133402832</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>0.04128910301268505</v>
+        <v>0.06416323848994489</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>25591.4</v>
+        <v>36262.7</v>
       </c>
       <c r="L4" s="6" t="n">
         <v>1</v>
@@ -6039,7 +6039,7 @@
         <v>58365.8</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>0.1240939119923837</v>
+        <v>0.1240939119923838</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>0.139350481130204</v>
@@ -6070,7 +6070,7 @@
         <v>182535.6</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>0.4918008330306788</v>
+        <v>0.491800833030679</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>147075.1</v>
@@ -6079,10 +6079,10 @@
         <v>35460.5</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>0.09554024486662686</v>
+        <v>0.095540244866627</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>0.08466317255083548</v>
+        <v>0.0846631725508355</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>47224.5</v>
@@ -6110,7 +6110,7 @@
         <v>99940.2</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.3995121498677655</v>
+        <v>0.3995121498677656</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>87928.10000000001</v>
@@ -6119,10 +6119,10 @@
         <v>12012.1</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>0.04801846387587927</v>
+        <v>0.04801846387587938</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>0.02867929804487862</v>
+        <v>0.02867929804487865</v>
       </c>
       <c r="K7" s="8" t="n">
         <v>18453</v>
@@ -6159,10 +6159,10 @@
         <v>28288.9</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>0.1169197131316401</v>
+        <v>0.1169197131316402</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>0.06754079303828144</v>
+        <v>0.06754079303828141</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>36416.6</v>
@@ -6184,28 +6184,28 @@
         <v>188144.6</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>156095.4</v>
+        <v>136064.7</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>112213.9</v>
+        <v>147596.3</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.7844835738457887</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>80164.7</v>
+        <v>95516.39999999999</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>32049.2</v>
+        <v>52079.9</v>
       </c>
       <c r="I9" s="23" t="n">
-        <v>0.1703432331211979</v>
+        <v>0.2768079740720661</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.07651850178172413</v>
+        <v>0.1243426643320709</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>39281.1</v>
+        <v>61592.2</v>
       </c>
       <c r="L9" s="9" t="n">
         <v>6</v>
@@ -6242,7 +6242,7 @@
         <v>-0.03833060178176359</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>-0.01546135175113704</v>
+        <v>-0.01546135175113701</v>
       </c>
       <c r="K10" s="5" t="n">
         <v>-3229.4</v>
@@ -6264,28 +6264,28 @@
         <v>150153</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>125401</v>
+        <v>109415</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>89554.8</v>
+        <v>117792.6</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.596423561408461</v>
+        <v>0.7844835738457887</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>64802.7</v>
+        <v>77054.5</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>24752.1</v>
+        <v>40738.1</v>
       </c>
       <c r="I11" s="23" t="n">
-        <v>0.1648457545474006</v>
+        <v>0.2713104954982688</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>0.05909650237926547</v>
+        <v>0.09726365951464501</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>30523.7</v>
+        <v>48329.6</v>
       </c>
       <c r="L11" s="9" t="n">
         <v>8</v>
@@ -6304,28 +6304,28 @@
         <v>135545.8</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>98404.89999999999</v>
+        <v>83974.10000000001</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>80842.7</v>
+        <v>106333.5</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.7844835738457887</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>43701.8</v>
+        <v>54761.7</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>37140.9</v>
+        <v>51571.8</v>
       </c>
       <c r="I12" s="22" t="n">
-        <v>0.2740099872223644</v>
+        <v>0.3804747281732325</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>0.08867524940395671</v>
+        <v>0.1231294222326443</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>42351.1</v>
+        <v>58424.7</v>
       </c>
       <c r="L12" s="6" t="n">
         <v>9</v>
@@ -6359,10 +6359,10 @@
         <v>14299.1</v>
       </c>
       <c r="I13" s="23" t="n">
-        <v>0.111416596622134</v>
+        <v>0.1114165966221341</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.03413959048977283</v>
+        <v>0.03413959048977282</v>
       </c>
       <c r="K13" s="8" t="n">
         <v>18360.9</v>
@@ -6384,28 +6384,28 @@
         <v>128178.4</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>103635</v>
+        <v>120524.2</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>79816</v>
+        <v>49982.6</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>0.6226945373212424</v>
+        <v>0.3899459584804174</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>55272.6</v>
+        <v>42328.5</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>24543.4</v>
+        <v>7654.1</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>0.1914784958652868</v>
+        <v>0.05971461458175745</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>0.05859824486873212</v>
+        <v>0.0182744886922738</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>29687.4</v>
+        <v>10875.4</v>
       </c>
       <c r="L14" s="6" t="n">
         <v>11</v>
@@ -6424,28 +6424,28 @@
         <v>99917.89999999999</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>81740.5</v>
+        <v>91293.8</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>56170.7</v>
+        <v>39295.7</v>
       </c>
       <c r="F15" s="10" t="n">
-        <v>0.5621684220927137</v>
+        <v>0.3932797405956895</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>37993.3</v>
+        <v>30671.6</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>18177.3</v>
+        <v>8624.1</v>
       </c>
       <c r="I15" s="23" t="n">
-        <v>0.1819228711815603</v>
+        <v>0.08631142517516095</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.04339906730708872</v>
+        <v>0.02059023874358925</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>21797.4</v>
+        <v>11156.6</v>
       </c>
       <c r="L15" s="9" t="n">
         <v>12</v>
@@ -6470,7 +6470,7 @@
         <v>43288</v>
       </c>
       <c r="F16" s="11" t="n">
-        <v>0.4639542338179102</v>
+        <v>0.4639542338179103</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>33943.9</v>
@@ -6479,7 +6479,7 @@
         <v>9344.1</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>0.1001488079826962</v>
+        <v>0.1001488079826963</v>
       </c>
       <c r="J16" s="11" t="n">
         <v>0.02230941938996182</v>
@@ -6519,10 +6519,10 @@
         <v>4536</v>
       </c>
       <c r="I17" s="23" t="n">
-        <v>0.05000563628186428</v>
+        <v>0.05000563628186443</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.01082996226462529</v>
+        <v>0.01082996226462531</v>
       </c>
       <c r="K17" s="8" t="n">
         <v>6673.9</v>
@@ -6544,28 +6544,28 @@
         <v>73384.39999999999</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>58177.8</v>
+        <v>50364.9</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>43768.2</v>
+        <v>57568.8</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.7844835738457887</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>28561.6</v>
+        <v>34549.4</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>15206.6</v>
+        <v>23019.5</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>0.2072185923549128</v>
+        <v>0.3136833333057809</v>
       </c>
       <c r="J18" s="11" t="n">
-        <v>0.03630631699499465</v>
+        <v>0.05495977173486586</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>18027.4</v>
+        <v>26729.6</v>
       </c>
       <c r="L18" s="6" t="n">
         <v>15</v>
@@ -6584,28 +6584,28 @@
         <v>60383.2</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>42979.4</v>
+        <v>61126.8</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>36014</v>
+        <v>3958.3</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.06555351510288186</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>18610.2</v>
+        <v>4701.9</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>17403.8</v>
-      </c>
-      <c r="I19" s="23" t="n">
-        <v>0.2882226909764236</v>
+        <v>-743.6</v>
+      </c>
+      <c r="I19" s="25" t="n">
+        <v>-0.01231404315430572</v>
       </c>
       <c r="J19" s="10" t="n">
-        <v>0.04155221307902743</v>
+        <v>-0.001775279188736408</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>19724.8</v>
+        <v>-488.5</v>
       </c>
       <c r="L19" s="9" t="n">
         <v>16</v>
@@ -6624,28 +6624,28 @@
         <v>59558.9</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>43330.6</v>
+        <v>36989.7</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>35522.3</v>
+        <v>46723</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.7844835738457886</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>19294</v>
+        <v>24153.8</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>16228.3</v>
+        <v>22569.2</v>
       </c>
       <c r="I20" s="22" t="n">
-        <v>0.2724748606340722</v>
+        <v>0.3789396015849404</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>0.03874564911913801</v>
+        <v>0.05388482741559775</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>18517.6</v>
+        <v>25580.4</v>
       </c>
       <c r="L20" s="6" t="n">
         <v>17</v>
@@ -6664,28 +6664,28 @@
         <v>58634.9</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>42513.3</v>
+        <v>57937.9</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>34971.3</v>
+        <v>7725.2</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.1317509470238122</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>18849.7</v>
+        <v>7028.2</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>16121.6</v>
+        <v>697</v>
       </c>
       <c r="I21" s="23" t="n">
-        <v>0.274948654420774</v>
+        <v>0.0118876832113264</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>0.03849088928700726</v>
+        <v>0.001664192535621323</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>18375.4</v>
+        <v>1194.9</v>
       </c>
       <c r="L21" s="9" t="n">
         <v>18</v>
@@ -6722,7 +6722,7 @@
         <v>0.08000340682931713</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>0.01092982966444593</v>
+        <v>0.01092982966444592</v>
       </c>
       <c r="K22" s="5" t="n">
         <v>5721.3</v>
@@ -6744,28 +6744,28 @@
         <v>56258.6</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46333.6</v>
+        <v>52522.3</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>32800.9</v>
+        <v>21869.2</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>0.5830381552047685</v>
+        <v>0.3887270638017194</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>22875.9</v>
+        <v>18132.9</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>9925</v>
+        <v>3736.3</v>
       </c>
       <c r="I23" s="23" t="n">
-        <v>0.1764169657560837</v>
+        <v>0.06641335711014552</v>
       </c>
       <c r="J23" s="10" t="n">
-        <v>0.02369621577862736</v>
+        <v>0.008920600317097176</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>12038.9</v>
+        <v>5145.7</v>
       </c>
       <c r="L23" s="9" t="n">
         <v>20</v>
@@ -6790,7 +6790,7 @@
         <v>12886.9</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>0.2931956292110319</v>
+        <v>0.293195629211032</v>
       </c>
       <c r="G24" s="5" t="n">
         <v>9950.4</v>
@@ -6799,10 +6799,10 @@
         <v>2936.5</v>
       </c>
       <c r="I24" s="22" t="n">
-        <v>0.06680929068011951</v>
+        <v>0.06680929068011966</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>0.007010959987568385</v>
+        <v>0.007010959987568391</v>
       </c>
       <c r="K24" s="5" t="n">
         <v>3767</v>
@@ -6824,28 +6824,28 @@
         <v>39033.7</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>36007.3</v>
+        <v>35446.1</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>11098.5</v>
+        <v>12089.8</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>0.2843299447747481</v>
+        <v>0.3097264024548309</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>8072</v>
+        <v>8502.1</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>3026.5</v>
+        <v>3587.7</v>
       </c>
       <c r="I25" s="23" t="n">
-        <v>0.07753451526892352</v>
+        <v>0.09191198580578622</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>0.007225781747504662</v>
+        <v>0.008565681324102478</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>3741.7</v>
+        <v>4366.8</v>
       </c>
       <c r="L25" s="9" t="n">
         <v>22</v>
@@ -6864,28 +6864,28 @@
         <v>38090.7</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>30072.2</v>
+        <v>33519.9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>21607.1</v>
+        <v>15517.1</v>
       </c>
       <c r="F26" s="11" t="n">
-        <v>0.5672537450322775</v>
+        <v>0.4073722024981647</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>13588.6</v>
+        <v>10946.3</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>8018.5</v>
+        <v>4570.8</v>
       </c>
       <c r="I26" s="22" t="n">
-        <v>0.2105100223756378</v>
+        <v>0.1199977077792954</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>0.01914439289545739</v>
+        <v>0.01091294009831892</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>9411</v>
+        <v>5570.8</v>
       </c>
       <c r="L26" s="6" t="n">
         <v>23</v>
@@ -6904,28 +6904,28 @@
         <v>31500</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>24226.5</v>
+        <v>27238.2</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>19350.2</v>
+        <v>14030.2</v>
       </c>
       <c r="F27" s="10" t="n">
-        <v>0.6142901955485539</v>
+        <v>0.4454015140515296</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>12076.6</v>
+        <v>9768.4</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>7273.6</v>
+        <v>4261.8</v>
       </c>
       <c r="I27" s="23" t="n">
-        <v>0.2309061831256214</v>
+        <v>0.135294737119222</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.01736586848857456</v>
+        <v>0.01017517409107426</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>8520.6</v>
+        <v>5166</v>
       </c>
       <c r="L27" s="9" t="n">
         <v>24</v>
@@ -6950,7 +6950,7 @@
         <v>10979.3</v>
       </c>
       <c r="F28" s="11" t="n">
-        <v>0.4145199878696137</v>
+        <v>0.4145199878696139</v>
       </c>
       <c r="G28" s="5" t="n">
         <v>10188.3</v>
@@ -6959,10 +6959,10 @@
         <v>791</v>
       </c>
       <c r="I28" s="22" t="n">
-        <v>0.02986494316823235</v>
+        <v>0.02986494316823248</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>0.001888609921246565</v>
+        <v>0.001888609921246571</v>
       </c>
       <c r="K28" s="5" t="n">
         <v>1498.6</v>
@@ -6999,10 +6999,10 @@
         <v>1586.3</v>
       </c>
       <c r="I29" s="23" t="n">
-        <v>0.06195977406014861</v>
+        <v>0.06195977406014876</v>
       </c>
       <c r="J29" s="10" t="n">
-        <v>0.00378733449818604</v>
+        <v>0.003787334498186043</v>
       </c>
       <c r="K29" s="8" t="n">
         <v>2054.4</v>
@@ -7042,7 +7042,7 @@
         <v>0.0378466262058419</v>
       </c>
       <c r="J30" s="11" t="n">
-        <v>0.002163156535879086</v>
+        <v>0.002163156535879083</v>
       </c>
       <c r="K30" s="5" t="n">
         <v>1263.3</v>
@@ -7079,10 +7079,10 @@
         <v>-595.8</v>
       </c>
       <c r="I31" s="25" t="n">
-        <v>-0.03667857655024201</v>
+        <v>-0.03667857655024189</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>-0.001422528774472499</v>
+        <v>-0.001422528774472492</v>
       </c>
       <c r="K31" s="8" t="n">
         <v>-184.5</v>
@@ -7104,28 +7104,28 @@
         <v>9136.5</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>8439.799999999999</v>
+        <v>8313.9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>2521.1</v>
+        <v>2743.5</v>
       </c>
       <c r="F32" s="11" t="n">
-        <v>0.2759387359155784</v>
+        <v>0.3002783652409303</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>1824.4</v>
+        <v>1920.9</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>696.7</v>
+        <v>822.6</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>0.07625589344312307</v>
+        <v>0.09003507115017191</v>
       </c>
       <c r="J32" s="11" t="n">
-        <v>0.001663429079303881</v>
+        <v>0.001964004993530058</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>859.2</v>
+        <v>999.4</v>
       </c>
       <c r="L32" s="6" t="n">
         <v>29</v>
@@ -7144,28 +7144,28 @@
         <v>8834.200000000001</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>6249.2</v>
+        <v>9211.299999999999</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>5268.9</v>
+        <v>36.7</v>
       </c>
       <c r="F33" s="10" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.004152356381903834</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>2683.9</v>
+        <v>413.8</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>2585</v>
-      </c>
-      <c r="I33" s="23" t="n">
-        <v>0.2926126019262937</v>
+        <v>-377.1</v>
+      </c>
+      <c r="I33" s="25" t="n">
+        <v>-0.04268462366984266</v>
       </c>
       <c r="J33" s="10" t="n">
-        <v>0.006171763271374426</v>
+        <v>-0.0009003009128237473</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>2924.6</v>
+        <v>-374.7</v>
       </c>
       <c r="L33" s="9" t="n">
         <v>30</v>
@@ -7199,10 +7199,10 @@
         <v>472.8</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>0.0687592874158507</v>
+        <v>0.06875928741585083</v>
       </c>
       <c r="J34" s="11" t="n">
-        <v>0.001128891587859104</v>
+        <v>0.001128891587859105</v>
       </c>
       <c r="K34" s="5" t="n">
         <v>591.9</v>
@@ -7224,28 +7224,28 @@
         <v>6748.3</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>4936.8</v>
+        <v>4218.3</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>4024.8</v>
+        <v>5293.9</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>0.596423561408461</v>
+        <v>0.7844835738457886</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>2213.3</v>
+        <v>2764</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>1811.5</v>
+        <v>2529.9</v>
       </c>
       <c r="I35" s="23" t="n">
-        <v>0.2684387827582595</v>
+        <v>0.3749035237091277</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.004325012466985357</v>
+        <v>0.006040343341218736</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>2070.9</v>
+        <v>2871.1</v>
       </c>
       <c r="L35" s="9" t="n">
         <v>32</v>
@@ -7264,28 +7264,28 @@
         <v>348.3</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>265.3</v>
+        <v>228.2</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>207.7</v>
+        <v>273.2</v>
       </c>
       <c r="F36" s="11" t="n">
-        <v>0.5964235614084609</v>
+        <v>0.7844835738457886</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>124.7</v>
+        <v>153.1</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>83</v>
+        <v>120.1</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>0.2383199732058857</v>
+        <v>0.344784714156754</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>0.000198180460418223</v>
+        <v>0.0002867136668302684</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>96.40000000000001</v>
+        <v>137.7</v>
       </c>
       <c r="L36" s="6" t="n">
         <v>33</v>
@@ -7421,7 +7421,7 @@
         <v>0.1557275848095814</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>92.3</v>
+        <v>102.83</v>
       </c>
       <c r="J4" s="20" t="inlineStr">
         <is>
@@ -7497,7 +7497,7 @@
         <v>371157.6</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>0.0991929963975428</v>
+        <v>0.09919299639754281</v>
       </c>
       <c r="H6" s="11" t="n">
         <v>0.3806192903694026</v>
@@ -7538,7 +7538,7 @@
         <v>250155.7</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>0.066854874139209</v>
+        <v>0.06685487413920901</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>0.4474741645086115</v>
@@ -7579,7 +7579,7 @@
         <v>241951.6</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>0.06466231300320691</v>
+        <v>0.06466231300320692</v>
       </c>
       <c r="H8" s="11" t="n">
         <v>0.5121364775118185</v>
@@ -7620,13 +7620,13 @@
         <v>188144.6</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>0.05028221411743813</v>
+        <v>0.05028221411743815</v>
       </c>
       <c r="H9" s="10" t="n">
         <v>0.5624186916292566</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>34.74</v>
+        <v>45.11</v>
       </c>
       <c r="J9" s="20" t="inlineStr">
         <is>
@@ -7702,13 +7702,13 @@
         <v>150153</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>0.04012886091449489</v>
+        <v>0.0401288609144949</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>0.6476993084190383</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>37.84</v>
+        <v>49.14</v>
       </c>
       <c r="J11" s="20" t="inlineStr">
         <is>
@@ -7743,13 +7743,13 @@
         <v>135545.8</v>
       </c>
       <c r="G12" s="11" t="n">
-        <v>0.03622503778477</v>
+        <v>0.03622503778477001</v>
       </c>
       <c r="H12" s="11" t="n">
         <v>0.6839243462038084</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>91.33</v>
+        <v>118.6</v>
       </c>
       <c r="J12" s="20" t="inlineStr">
         <is>
@@ -7831,7 +7831,7 @@
         <v>0.7524793898733501</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>234.98</v>
+        <v>151.65</v>
       </c>
       <c r="J14" s="20" t="inlineStr">
         <is>
@@ -7872,7 +7872,7 @@
         <v>0.7791827501675835</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>17.64</v>
+        <v>12.64</v>
       </c>
       <c r="J15" s="20" t="inlineStr">
         <is>
@@ -7995,7 +7995,7 @@
         <v>0.8479729799175554</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>278.52</v>
+        <v>361.65</v>
       </c>
       <c r="J18" s="27" t="inlineStr">
         <is>
@@ -8036,7 +8036,7 @@
         <v>0.8641105749084409</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>58.8</v>
+        <v>9.25</v>
       </c>
       <c r="J19" s="27" t="inlineStr">
         <is>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="K19" s="26" t="inlineStr">
         <is>
-          <t>تثبيت</t>
+          <t>رفع السعر</t>
         </is>
       </c>
     </row>
@@ -8077,7 +8077,7 @@
         <v>0.8800278720250037</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>100.33</v>
+        <v>130.28</v>
       </c>
       <c r="J20" s="27" t="inlineStr">
         <is>
@@ -8118,7 +8118,7 @@
         <v>0.8956982390124839</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>46.35</v>
+        <v>12.16</v>
       </c>
       <c r="J21" s="27" t="inlineStr">
         <is>
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K21" s="26" t="inlineStr">
         <is>
-          <t>تثبيت</t>
+          <t>رفع السعر</t>
         </is>
       </c>
     </row>
@@ -8194,13 +8194,13 @@
         <v>56258.6</v>
       </c>
       <c r="G23" s="10" t="n">
-        <v>0.01503527820941494</v>
+        <v>0.01503527820941495</v>
       </c>
       <c r="H23" s="10" t="n">
         <v>0.9260259906139299</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>37.02</v>
+        <v>25.36</v>
       </c>
       <c r="J23" s="27" t="inlineStr">
         <is>
@@ -8209,7 +8209,7 @@
       </c>
       <c r="K23" s="26" t="inlineStr">
         <is>
-          <t>تثبيت</t>
+          <t>رفع السعر</t>
         </is>
       </c>
     </row>
@@ -8282,7 +8282,7 @@
         <v>0.9482045049679356</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>35.16</v>
+        <v>37.96</v>
       </c>
       <c r="J25" s="27" t="inlineStr">
         <is>
@@ -8323,7 +8323,7 @@
         <v>0.9583843611428484</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>18.79</v>
+        <v>13.79</v>
       </c>
       <c r="J26" s="28" t="inlineStr">
         <is>
@@ -8364,7 +8364,7 @@
         <v>0.9668028427289416</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>44.76</v>
+        <v>33.09</v>
       </c>
       <c r="J27" s="28" t="inlineStr">
         <is>
@@ -8399,7 +8399,7 @@
         <v>26486.9</v>
       </c>
       <c r="G28" s="11" t="n">
-        <v>0.007078698175775099</v>
+        <v>0.0070786981757751</v>
       </c>
       <c r="H28" s="11" t="n">
         <v>0.9738815409047167</v>
@@ -8563,13 +8563,13 @@
         <v>9136.5</v>
       </c>
       <c r="G32" s="11" t="n">
-        <v>0.002441764056534443</v>
+        <v>0.002441764056534444</v>
       </c>
       <c r="H32" s="11" t="n">
         <v>0.9939046784388077</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>15.62</v>
+        <v>16.85</v>
       </c>
       <c r="J32" s="28" t="inlineStr">
         <is>
@@ -8604,13 +8604,13 @@
         <v>8834.200000000001</v>
       </c>
       <c r="G33" s="10" t="n">
-        <v>0.002360962312724731</v>
+        <v>0.002360962312724732</v>
       </c>
       <c r="H33" s="10" t="n">
         <v>0.9962656407515323</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>161.33</v>
+        <v>9.67</v>
       </c>
       <c r="J33" s="28" t="inlineStr">
         <is>
@@ -8619,7 +8619,7 @@
       </c>
       <c r="K33" s="26" t="inlineStr">
         <is>
-          <t>تثبيت</t>
+          <t>رفع السعر</t>
         </is>
       </c>
     </row>
@@ -8692,7 +8692,7 @@
         <v>0.9999069163911312</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>94.48</v>
+        <v>122.68</v>
       </c>
       <c r="J35" s="28" t="inlineStr">
         <is>
@@ -8727,13 +8727,13 @@
         <v>348.3</v>
       </c>
       <c r="G36" s="11" t="n">
-        <v>9.308360886878802e-05</v>
+        <v>9.308360886878803e-05</v>
       </c>
       <c r="H36" s="11" t="n">
         <v>1</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>73.15000000000001</v>
+        <v>94.98</v>
       </c>
       <c r="J36" s="28" t="inlineStr">
         <is>
@@ -8913,40 +8913,40 @@
         <v>374.78</v>
       </c>
       <c r="F4" s="33" t="n">
-        <v>399.75</v>
+        <v>393</v>
       </c>
       <c r="G4" s="32" t="n">
-        <v>24.97</v>
+        <v>18.22</v>
       </c>
       <c r="H4" s="34" t="n">
-        <v>0.06661948445477561</v>
+        <v>0.04860902411689016</v>
       </c>
       <c r="I4" s="32" t="n">
-        <v>273.25</v>
+        <v>262.72</v>
       </c>
       <c r="J4" s="32" t="n">
         <v>9.23</v>
       </c>
       <c r="K4" s="32" t="n">
-        <v>38.83</v>
+        <v>38.67</v>
       </c>
       <c r="L4" s="32" t="n">
-        <v>321.31</v>
+        <v>310.62</v>
       </c>
       <c r="M4" s="32" t="n">
-        <v>317.08</v>
+        <v>306.54</v>
       </c>
       <c r="N4" s="32" t="n">
-        <v>34.76</v>
+        <v>39.33</v>
       </c>
       <c r="O4" s="32" t="n">
-        <v>351.84</v>
+        <v>345.88</v>
       </c>
       <c r="P4" s="32" t="n">
-        <v>399.82</v>
+        <v>393.04</v>
       </c>
       <c r="Q4" s="35" t="n">
-        <v>0.1198551532679202</v>
+        <v>0.1199081903669368</v>
       </c>
       <c r="R4" s="36" t="inlineStr">
         <is>
@@ -9010,7 +9010,7 @@
         <v>52.11</v>
       </c>
       <c r="Q5" s="41" t="n">
-        <v>0.151130217610674</v>
+        <v>0.1511302176106741</v>
       </c>
       <c r="R5" s="42" t="inlineStr">
         <is>
@@ -9242,31 +9242,31 @@
         <v>9.256116750488985e-05</v>
       </c>
       <c r="I9" s="39" t="n">
-        <v>22.25</v>
+        <v>11.88</v>
       </c>
       <c r="J9" s="39" t="n">
         <v>0</v>
       </c>
       <c r="K9" s="39" t="n">
-        <v>9.56</v>
+        <v>9.4</v>
       </c>
       <c r="L9" s="39" t="n">
-        <v>31.81</v>
+        <v>21.29</v>
       </c>
       <c r="M9" s="39" t="n">
-        <v>31.48</v>
+        <v>21.11</v>
       </c>
       <c r="N9" s="39" t="n">
-        <v>14.27</v>
+        <v>18.77</v>
       </c>
       <c r="O9" s="39" t="n">
-        <v>45.75</v>
+        <v>39.88</v>
       </c>
       <c r="P9" s="39" t="n">
-        <v>50.27</v>
+        <v>43.82</v>
       </c>
       <c r="Q9" s="41" t="n">
-        <v>0.1973868046684868</v>
+        <v>0.3003812107120655</v>
       </c>
       <c r="R9" s="42" t="inlineStr">
         <is>
@@ -9370,31 +9370,31 @@
         <v>-0.001275789636464353</v>
       </c>
       <c r="I11" s="39" t="n">
-        <v>24.24</v>
+        <v>12.94</v>
       </c>
       <c r="J11" s="39" t="n">
         <v>0</v>
       </c>
       <c r="K11" s="39" t="n">
-        <v>10.74</v>
+        <v>10.57</v>
       </c>
       <c r="L11" s="39" t="n">
-        <v>34.98</v>
+        <v>23.52</v>
       </c>
       <c r="M11" s="39" t="n">
-        <v>34.62</v>
+        <v>23.32</v>
       </c>
       <c r="N11" s="39" t="n">
-        <v>15.54</v>
+        <v>20.44</v>
       </c>
       <c r="O11" s="39" t="n">
-        <v>50.16</v>
+        <v>43.77</v>
       </c>
       <c r="P11" s="39" t="n">
-        <v>54.52</v>
+        <v>47.57</v>
       </c>
       <c r="Q11" s="41" t="n">
-        <v>0.1909615765165464</v>
+        <v>0.2940970950683147</v>
       </c>
       <c r="R11" s="42" t="inlineStr">
         <is>
@@ -9434,31 +9434,31 @@
         <v>-0.0005977872947894314</v>
       </c>
       <c r="I12" s="32" t="n">
-        <v>58.51</v>
+        <v>31.24</v>
       </c>
       <c r="J12" s="32" t="n">
         <v>0</v>
       </c>
       <c r="K12" s="32" t="n">
-        <v>10.1</v>
+        <v>9.69</v>
       </c>
       <c r="L12" s="32" t="n">
-        <v>68.61</v>
+        <v>40.94</v>
       </c>
       <c r="M12" s="32" t="n">
-        <v>67.73</v>
+        <v>40.47</v>
       </c>
       <c r="N12" s="32" t="n">
-        <v>37.51</v>
+        <v>49.34</v>
       </c>
       <c r="O12" s="32" t="n">
-        <v>105.25</v>
+        <v>89.81</v>
       </c>
       <c r="P12" s="32" t="n">
-        <v>116.94</v>
+        <v>99.79000000000001</v>
       </c>
       <c r="Q12" s="35" t="n">
-        <v>0.2971892879207779</v>
+        <v>0.4002548385235071</v>
       </c>
       <c r="R12" s="42" t="inlineStr">
         <is>
@@ -9553,40 +9553,40 @@
         <v>370.07</v>
       </c>
       <c r="F14" s="33" t="n">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="G14" s="32" t="n">
-        <v>-0.07000000000000001</v>
+        <v>3.93</v>
       </c>
       <c r="H14" s="41" t="n">
-        <v>-0.0001887006076158881</v>
+        <v>0.01062007019662614</v>
       </c>
       <c r="I14" s="32" t="n">
-        <v>119.03</v>
+        <v>202.36</v>
       </c>
       <c r="J14" s="32" t="n">
         <v>16.06</v>
       </c>
       <c r="K14" s="32" t="n">
-        <v>59.69</v>
+        <v>60.94</v>
       </c>
       <c r="L14" s="32" t="n">
-        <v>194.78</v>
+        <v>279.36</v>
       </c>
       <c r="M14" s="32" t="n">
-        <v>192.75</v>
+        <v>276.08</v>
       </c>
       <c r="N14" s="32" t="n">
-        <v>96.73</v>
+        <v>60.58</v>
       </c>
       <c r="O14" s="32" t="n">
-        <v>289.48</v>
+        <v>336.66</v>
       </c>
       <c r="P14" s="32" t="n">
-        <v>321.65</v>
+        <v>374.07</v>
       </c>
       <c r="Q14" s="35" t="n">
-        <v>0.2176131052008912</v>
+        <v>0.09983981459945633</v>
       </c>
       <c r="R14" s="42" t="inlineStr">
         <is>
@@ -9626,31 +9626,31 @@
         <v>-0.00326797385620925</v>
       </c>
       <c r="I15" s="39" t="n">
-        <v>8.33</v>
+        <v>13.33</v>
       </c>
       <c r="J15" s="39" t="n">
         <v>4.63</v>
       </c>
       <c r="K15" s="39" t="n">
-        <v>4.23</v>
+        <v>4.31</v>
       </c>
       <c r="L15" s="39" t="n">
-        <v>17.19</v>
+        <v>22.27</v>
       </c>
       <c r="M15" s="39" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N15" s="39" t="n">
-        <v>7.22</v>
+        <v>5.05</v>
       </c>
       <c r="O15" s="39" t="n">
-        <v>24.22</v>
+        <v>27.05</v>
       </c>
       <c r="P15" s="39" t="n">
-        <v>26.91</v>
+        <v>30.06</v>
       </c>
       <c r="Q15" s="41" t="n">
-        <v>0.2059207074412663</v>
+        <v>0.1131139698724799</v>
       </c>
       <c r="R15" s="42" t="inlineStr">
         <is>
@@ -9818,31 +9818,31 @@
         <v>0.0001582069874752623</v>
       </c>
       <c r="I18" s="32" t="n">
-        <v>178.41</v>
+        <v>95.27</v>
       </c>
       <c r="J18" s="32" t="n">
         <v>0</v>
       </c>
       <c r="K18" s="32" t="n">
-        <v>60.34</v>
+        <v>59.09</v>
       </c>
       <c r="L18" s="32" t="n">
-        <v>238.75</v>
+        <v>154.36</v>
       </c>
       <c r="M18" s="32" t="n">
-        <v>236.07</v>
+        <v>152.93</v>
       </c>
       <c r="N18" s="32" t="n">
-        <v>114.4</v>
+        <v>150.47</v>
       </c>
       <c r="O18" s="32" t="n">
-        <v>350.47</v>
+        <v>303.4</v>
       </c>
       <c r="P18" s="32" t="n">
-        <v>393.78</v>
+        <v>340.9</v>
       </c>
       <c r="Q18" s="35" t="n">
-        <v>0.233110509585868</v>
+        <v>0.336098155546702</v>
       </c>
       <c r="R18" s="42" t="inlineStr">
         <is>
@@ -9873,44 +9873,44 @@
         <v>96.45999999999999</v>
       </c>
       <c r="F19" s="40" t="n">
-        <v>96.5</v>
+        <v>109.75</v>
       </c>
       <c r="G19" s="39" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="H19" s="41" t="n">
-        <v>0.0003765301544573774</v>
+        <v>13.29</v>
+      </c>
+      <c r="H19" s="34" t="n">
+        <v>0.1377339293725566</v>
       </c>
       <c r="I19" s="39" t="n">
-        <v>37.66</v>
+        <v>80.95999999999999</v>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="K19" s="39" t="n">
-        <v>5.18</v>
+        <v>5.92</v>
       </c>
       <c r="L19" s="39" t="n">
-        <v>42.84</v>
+        <v>93.13</v>
       </c>
       <c r="M19" s="39" t="n">
-        <v>42.28</v>
+        <v>91.81999999999999</v>
       </c>
       <c r="N19" s="39" t="n">
-        <v>24.15</v>
+        <v>2.65</v>
       </c>
       <c r="O19" s="39" t="n">
-        <v>66.43000000000001</v>
+        <v>94.48</v>
       </c>
       <c r="P19" s="39" t="n">
-        <v>77.23999999999999</v>
+        <v>109.86</v>
       </c>
       <c r="Q19" s="41" t="n">
-        <v>0.3116193130836326</v>
-      </c>
-      <c r="R19" s="42" t="inlineStr">
-        <is>
-          <t>تثبيت</t>
+        <v>0.1391597113267514</v>
+      </c>
+      <c r="R19" s="36" t="inlineStr">
+        <is>
+          <t>رفع السعر</t>
         </is>
       </c>
     </row>
@@ -9946,31 +9946,31 @@
         <v>-0.0006010396361273429</v>
       </c>
       <c r="I20" s="32" t="n">
-        <v>64.27</v>
+        <v>34.32</v>
       </c>
       <c r="J20" s="32" t="n">
         <v>0</v>
       </c>
       <c r="K20" s="32" t="n">
-        <v>11.34</v>
+        <v>10.89</v>
       </c>
       <c r="L20" s="32" t="n">
-        <v>75.61</v>
+        <v>45.21</v>
       </c>
       <c r="M20" s="32" t="n">
-        <v>74.65000000000001</v>
+        <v>44.7</v>
       </c>
       <c r="N20" s="32" t="n">
-        <v>41.21</v>
+        <v>54.2</v>
       </c>
       <c r="O20" s="32" t="n">
-        <v>115.86</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="P20" s="32" t="n">
-        <v>128.73</v>
+        <v>109.89</v>
       </c>
       <c r="Q20" s="35" t="n">
-        <v>0.2957008826336625</v>
+        <v>0.3987667686423348</v>
       </c>
       <c r="R20" s="42" t="inlineStr">
         <is>
@@ -10001,44 +10001,44 @@
         <v>76.04000000000001</v>
       </c>
       <c r="F21" s="40" t="n">
-        <v>76</v>
+        <v>84.5</v>
       </c>
       <c r="G21" s="39" t="n">
-        <v>-0.04</v>
-      </c>
-      <c r="H21" s="41" t="n">
-        <v>-0.0005445095289168256</v>
+        <v>8.460000000000001</v>
+      </c>
+      <c r="H21" s="34" t="n">
+        <v>0.1112366966421912</v>
       </c>
       <c r="I21" s="39" t="n">
-        <v>29.69</v>
+        <v>57.63</v>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="K21" s="39" t="n">
-        <v>5.06</v>
+        <v>5.57</v>
       </c>
       <c r="L21" s="39" t="n">
-        <v>34.75</v>
+        <v>69.45</v>
       </c>
       <c r="M21" s="39" t="n">
-        <v>34.3</v>
+        <v>68.48999999999999</v>
       </c>
       <c r="N21" s="39" t="n">
-        <v>19.04</v>
+        <v>4.21</v>
       </c>
       <c r="O21" s="39" t="n">
-        <v>53.34</v>
+        <v>72.69</v>
       </c>
       <c r="P21" s="39" t="n">
-        <v>62.03</v>
+        <v>84.53</v>
       </c>
       <c r="Q21" s="41" t="n">
-        <v>0.2981354016377122</v>
-      </c>
-      <c r="R21" s="42" t="inlineStr">
-        <is>
-          <t>تثبيت</t>
+        <v>0.1397042633751014</v>
+      </c>
+      <c r="R21" s="36" t="inlineStr">
+        <is>
+          <t>رفع السعر</t>
         </is>
       </c>
     </row>
@@ -10129,44 +10129,44 @@
         <v>62.06</v>
       </c>
       <c r="F23" s="40" t="n">
-        <v>62</v>
+        <v>63.75</v>
       </c>
       <c r="G23" s="39" t="n">
-        <v>-0.06</v>
-      </c>
-      <c r="H23" s="41" t="n">
-        <v>-0.0009424098175713214</v>
+        <v>1.69</v>
+      </c>
+      <c r="H23" s="34" t="n">
+        <v>0.02725679635693279</v>
       </c>
       <c r="I23" s="39" t="n">
-        <v>19.04</v>
+        <v>30.71</v>
       </c>
       <c r="J23" s="39" t="n">
         <v>5.99</v>
       </c>
       <c r="K23" s="39" t="n">
-        <v>9.6</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="L23" s="39" t="n">
-        <v>34.64</v>
+        <v>46.48</v>
       </c>
       <c r="M23" s="39" t="n">
-        <v>34.26</v>
+        <v>45.93</v>
       </c>
       <c r="N23" s="39" t="n">
-        <v>15.19</v>
+        <v>10.13</v>
       </c>
       <c r="O23" s="39" t="n">
-        <v>49.45</v>
+        <v>56.05</v>
       </c>
       <c r="P23" s="39" t="n">
-        <v>56.19</v>
+        <v>63.7</v>
       </c>
       <c r="Q23" s="41" t="n">
-        <v>0.2024371793516645</v>
-      </c>
-      <c r="R23" s="42" t="inlineStr">
-        <is>
-          <t>تثبيت</t>
+        <v>0.1207271994168559</v>
+      </c>
+      <c r="R23" s="36" t="inlineStr">
+        <is>
+          <t>رفع السعر</t>
         </is>
       </c>
     </row>
@@ -10257,40 +10257,40 @@
         <v>114.29</v>
       </c>
       <c r="F25" s="40" t="n">
-        <v>118.5</v>
+        <v>116.75</v>
       </c>
       <c r="G25" s="39" t="n">
-        <v>4.21</v>
+        <v>2.46</v>
       </c>
       <c r="H25" s="34" t="n">
-        <v>0.03681478837631258</v>
+        <v>0.0215031775775063</v>
       </c>
       <c r="I25" s="39" t="n">
-        <v>72.87</v>
+        <v>70.06</v>
       </c>
       <c r="J25" s="39" t="n">
         <v>6.27</v>
       </c>
       <c r="K25" s="39" t="n">
-        <v>10.41</v>
+        <v>10.37</v>
       </c>
       <c r="L25" s="39" t="n">
-        <v>89.55</v>
+        <v>86.7</v>
       </c>
       <c r="M25" s="39" t="n">
-        <v>88.36</v>
+        <v>85.55</v>
       </c>
       <c r="N25" s="39" t="n">
-        <v>13.64</v>
+        <v>14.86</v>
       </c>
       <c r="O25" s="39" t="n">
-        <v>102</v>
+        <v>100.41</v>
       </c>
       <c r="P25" s="39" t="n">
-        <v>118.61</v>
+        <v>116.76</v>
       </c>
       <c r="Q25" s="41" t="n">
-        <v>0.1392104717233753</v>
+        <v>0.139925138426678</v>
       </c>
       <c r="R25" s="36" t="inlineStr">
         <is>
@@ -10330,31 +10330,31 @@
         <v>-0.002285975540061824</v>
       </c>
       <c r="I26" s="32" t="n">
-        <v>8.33</v>
+        <v>13.33</v>
       </c>
       <c r="J26" s="32" t="n">
         <v>5.2</v>
       </c>
       <c r="K26" s="32" t="n">
-        <v>3.66</v>
+        <v>3.74</v>
       </c>
       <c r="L26" s="32" t="n">
-        <v>17.2</v>
+        <v>22.27</v>
       </c>
       <c r="M26" s="32" t="n">
-        <v>16.99</v>
+        <v>21.99</v>
       </c>
       <c r="N26" s="32" t="n">
-        <v>7.7</v>
+        <v>5.53</v>
       </c>
       <c r="O26" s="32" t="n">
-        <v>24.69</v>
+        <v>27.52</v>
       </c>
       <c r="P26" s="32" t="n">
-        <v>28.38</v>
+        <v>31.63</v>
       </c>
       <c r="Q26" s="35" t="n">
-        <v>0.234423530205873</v>
+        <v>0.1466528171563232</v>
       </c>
       <c r="R26" s="42" t="inlineStr">
         <is>
@@ -10394,31 +10394,31 @@
         <v>0.001400560224089853</v>
       </c>
       <c r="I27" s="39" t="n">
-        <v>19.44</v>
+        <v>31.11</v>
       </c>
       <c r="J27" s="39" t="n">
         <v>7.2</v>
       </c>
       <c r="K27" s="39" t="n">
-        <v>8.470000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="L27" s="39" t="n">
-        <v>35.12</v>
+        <v>46.96</v>
       </c>
       <c r="M27" s="39" t="n">
-        <v>34.72</v>
+        <v>46.38</v>
       </c>
       <c r="N27" s="39" t="n">
-        <v>18.41</v>
+        <v>13.35</v>
       </c>
       <c r="O27" s="39" t="n">
-        <v>53.13</v>
+        <v>59.73</v>
       </c>
       <c r="P27" s="39" t="n">
-        <v>61.07</v>
+        <v>68.66</v>
       </c>
       <c r="Q27" s="41" t="n">
-        <v>0.2569474610128505</v>
+        <v>0.1645733888872752</v>
       </c>
       <c r="R27" s="42" t="inlineStr">
         <is>
@@ -10546,7 +10546,7 @@
         <v>132.12</v>
       </c>
       <c r="Q29" s="41" t="n">
-        <v>0.1692365203400157</v>
+        <v>0.169236520340016</v>
       </c>
       <c r="R29" s="36" t="inlineStr">
         <is>
@@ -10705,40 +10705,40 @@
         <v>52.17</v>
       </c>
       <c r="F32" s="33" t="n">
-        <v>56.25</v>
+        <v>55.25</v>
       </c>
       <c r="G32" s="32" t="n">
-        <v>4.08</v>
+        <v>3.08</v>
       </c>
       <c r="H32" s="34" t="n">
-        <v>0.07812251813416626</v>
+        <v>0.05895589558955883</v>
       </c>
       <c r="I32" s="32" t="n">
-        <v>31.88</v>
+        <v>30.65</v>
       </c>
       <c r="J32" s="32" t="n">
         <v>4.67</v>
       </c>
       <c r="K32" s="32" t="n">
-        <v>4.58</v>
+        <v>4.57</v>
       </c>
       <c r="L32" s="32" t="n">
-        <v>41.13</v>
+        <v>39.89</v>
       </c>
       <c r="M32" s="32" t="n">
-        <v>40.59</v>
+        <v>39.36</v>
       </c>
       <c r="N32" s="32" t="n">
-        <v>6.04</v>
+        <v>6.58</v>
       </c>
       <c r="O32" s="32" t="n">
-        <v>46.63</v>
+        <v>45.93</v>
       </c>
       <c r="P32" s="32" t="n">
-        <v>56.18</v>
+        <v>55.34</v>
       </c>
       <c r="Q32" s="35" t="n">
-        <v>0.1710437767476952</v>
+        <v>0.1686291087755525</v>
       </c>
       <c r="R32" s="36" t="inlineStr">
         <is>
@@ -10769,44 +10769,44 @@
         <v>264.67</v>
       </c>
       <c r="F33" s="40" t="n">
-        <v>264.75</v>
+        <v>310.5</v>
       </c>
       <c r="G33" s="39" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="H33" s="41" t="n">
-        <v>0.0003148614609571609</v>
+        <v>45.83</v>
+      </c>
+      <c r="H33" s="34" t="n">
+        <v>0.1731738035264483</v>
       </c>
       <c r="I33" s="39" t="n">
-        <v>103.34</v>
+        <v>253</v>
       </c>
       <c r="J33" s="39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K33" s="39" t="n">
-        <v>13.08</v>
+        <v>15.36</v>
       </c>
       <c r="L33" s="39" t="n">
-        <v>116.42</v>
+        <v>270.36</v>
       </c>
       <c r="M33" s="39" t="n">
-        <v>114.87</v>
+        <v>266.53</v>
       </c>
       <c r="N33" s="39" t="n">
-        <v>66.26000000000001</v>
+        <v>0.46</v>
       </c>
       <c r="O33" s="39" t="n">
-        <v>181.14</v>
+        <v>266.99</v>
       </c>
       <c r="P33" s="39" t="n">
-        <v>210.62</v>
+        <v>310.46</v>
       </c>
       <c r="Q33" s="41" t="n">
-        <v>0.315822748128182</v>
-      </c>
-      <c r="R33" s="42" t="inlineStr">
-        <is>
-          <t>تثبيت</t>
+        <v>0.1401184216468533</v>
+      </c>
+      <c r="R33" s="36" t="inlineStr">
+        <is>
+          <t>رفع السعر</t>
         </is>
       </c>
     </row>
@@ -10866,7 +10866,7 @@
         <v>54.33</v>
       </c>
       <c r="Q34" s="35" t="n">
-        <v>0.1687246950416877</v>
+        <v>0.1687246950416878</v>
       </c>
       <c r="R34" s="36" t="inlineStr">
         <is>
@@ -10906,31 +10906,31 @@
         <v>0</v>
       </c>
       <c r="I35" s="39" t="n">
-        <v>60.52</v>
+        <v>32.32</v>
       </c>
       <c r="J35" s="39" t="n">
         <v>0</v>
       </c>
       <c r="K35" s="39" t="n">
-        <v>11.29</v>
+        <v>10.86</v>
       </c>
       <c r="L35" s="39" t="n">
-        <v>71.81</v>
+        <v>43.18</v>
       </c>
       <c r="M35" s="39" t="n">
-        <v>70.90000000000001</v>
+        <v>42.7</v>
       </c>
       <c r="N35" s="39" t="n">
-        <v>38.81</v>
+        <v>51.04</v>
       </c>
       <c r="O35" s="39" t="n">
-        <v>109.71</v>
+        <v>93.73999999999999</v>
       </c>
       <c r="P35" s="39" t="n">
-        <v>129.07</v>
+        <v>110.28</v>
       </c>
       <c r="Q35" s="41" t="n">
-        <v>0.2922193154179272</v>
+        <v>0.3952232547439758</v>
       </c>
       <c r="R35" s="42" t="inlineStr">
         <is>
@@ -10970,31 +10970,31 @@
         <v>0</v>
       </c>
       <c r="I36" s="32" t="n">
-        <v>46.85</v>
+        <v>25.02</v>
       </c>
       <c r="J36" s="32" t="n">
         <v>0</v>
       </c>
       <c r="K36" s="32" t="n">
-        <v>12.23</v>
+        <v>11.91</v>
       </c>
       <c r="L36" s="32" t="n">
-        <v>59.09</v>
+        <v>36.93</v>
       </c>
       <c r="M36" s="32" t="n">
-        <v>58.39</v>
+        <v>36.55</v>
       </c>
       <c r="N36" s="32" t="n">
-        <v>30.04</v>
+        <v>39.52</v>
       </c>
       <c r="O36" s="32" t="n">
-        <v>88.43000000000001</v>
+        <v>76.06999999999999</v>
       </c>
       <c r="P36" s="32" t="n">
-        <v>104.04</v>
+        <v>89.48999999999999</v>
       </c>
       <c r="Q36" s="35" t="n">
-        <v>0.2630795645107493</v>
+        <v>0.3660835038367979</v>
       </c>
       <c r="R36" s="42" t="inlineStr">
         <is>
@@ -11017,7 +11017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11167,7 +11167,7 @@
         <v>0.12</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>0.02967855287448811</v>
+        <v>0.04612045133402832</v>
       </c>
       <c r="F10" s="44" t="inlineStr">
         <is>
@@ -11193,7 +11193,7 @@
         <v>0.08</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.04801846387587927</v>
+        <v>0.04801846387587938</v>
       </c>
       <c r="F11" s="44" t="inlineStr">
         <is>
@@ -11229,23 +11229,23 @@
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
-        <v>399</v>
+        <v>257</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>كفته اسبيشيال صغير</t>
+          <t>سجق الهنا 5 كيلو</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>0.05000563628186428</v>
+        <v>0.05971461458175745</v>
       </c>
       <c r="F13" s="44" t="inlineStr">
         <is>
@@ -11255,11 +11255,11 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>80</v>
+        <v>399</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>برجر 1200 جم</t>
+          <t>كفته اسبيشيال صغير</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -11268,10 +11268,10 @@
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>0.08000340682931713</v>
+        <v>0.05000563628186443</v>
       </c>
       <c r="F14" s="44" t="inlineStr">
         <is>
@@ -11281,11 +11281,11 @@
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
-        <v>255</v>
+        <v>1</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>برجر ابو هاشم جامبو 1.5 كيلو</t>
+          <t>مفروم صافي 400 جم (ابو هاشم)</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -11297,7 +11297,7 @@
         <v>0.14</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>0.06680929068011951</v>
+        <v>-0.01231404315430572</v>
       </c>
       <c r="F15" s="44" t="inlineStr">
         <is>
@@ -11307,11 +11307,11 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>107</v>
+        <v>2</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>سجق 800 ابو هاشم</t>
+          <t>كبده اسكندراني 400 (ابو هاشم)</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -11323,7 +11323,7 @@
         <v>0.14</v>
       </c>
       <c r="E16" s="11" t="n">
-        <v>0.07753451526892352</v>
+        <v>0.0118876832113264</v>
       </c>
       <c r="F16" s="44" t="inlineStr">
         <is>
@@ -11333,23 +11333,23 @@
     </row>
     <row r="17">
       <c r="A17" s="9" t="n">
-        <v>420</v>
+        <v>80</v>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>برجر الهنا 800 جرام</t>
+          <t>برجر 1200 جم</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D17" s="10" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>0.02986494316823235</v>
+        <v>0.08000340682931713</v>
       </c>
       <c r="F17" s="44" t="inlineStr">
         <is>
@@ -11359,23 +11359,23 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>421</v>
+        <v>99</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>برجر ابو هاشم 1 ك</t>
+          <t>سجق الهنا 800 جرام</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>0.06195977406014861</v>
+        <v>0.06641335711014552</v>
       </c>
       <c r="F18" s="44" t="inlineStr">
         <is>
@@ -11385,23 +11385,23 @@
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
-        <v>114</v>
+        <v>255</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>كفته ابو هاشم 800</t>
+          <t>برجر ابو هاشم جامبو 1.5 كيلو</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>0.17</v>
+        <v>0.14</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>0.0378466262058419</v>
+        <v>0.06680929068011966</v>
       </c>
       <c r="F19" s="44" t="inlineStr">
         <is>
@@ -11411,37 +11411,37 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>292</v>
+        <v>107</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>عجينه سجق 5 كيلو الهنا</t>
+          <t>سجق 800 ابو هاشم</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>-0.03667857655024201</v>
+        <v>0.09191198580578622</v>
       </c>
       <c r="F20" s="44" t="inlineStr">
         <is>
-          <t>بيع &lt; تكلفة محمّلة؛ هامش دون المستهدف</t>
+          <t>هامش دون المستهدف</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
-        <v>7</v>
+        <v>420</v>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>سجق 350 جم ابو هاشم</t>
+          <t>برجر الهنا 800 جرام</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -11450,10 +11450,10 @@
         </is>
       </c>
       <c r="D21" s="10" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>0.07625589344312307</v>
+        <v>0.02986494316823248</v>
       </c>
       <c r="F21" s="44" t="inlineStr">
         <is>
@@ -11463,11 +11463,11 @@
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>8</v>
+        <v>421</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>كفته 350 جم ابو هاشم</t>
+          <t>برجر ابو هاشم 1 ك</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -11479,9 +11479,139 @@
         <v>0.17</v>
       </c>
       <c r="E22" s="11" t="n">
-        <v>0.0687592874158507</v>
+        <v>0.06195977406014876</v>
       </c>
       <c r="F22" s="44" t="inlineStr">
+        <is>
+          <t>هامش دون المستهدف</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="n">
+        <v>114</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>كفته ابو هاشم 800</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>0.0378466262058419</v>
+      </c>
+      <c r="F23" s="44" t="inlineStr">
+        <is>
+          <t>هامش دون المستهدف</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>292</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>عجينه سجق 5 كيلو الهنا</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>-0.03667857655024189</v>
+      </c>
+      <c r="F24" s="44" t="inlineStr">
+        <is>
+          <t>بيع &lt; تكلفة محمّلة؛ هامش دون المستهدف</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>سجق 350 جم ابو هاشم</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>0.09003507115017191</v>
+      </c>
+      <c r="F25" s="44" t="inlineStr">
+        <is>
+          <t>هامش دون المستهدف</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>كيلو مفروم هندي</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <v>-0.04268462366984266</v>
+      </c>
+      <c r="F26" s="44" t="inlineStr">
+        <is>
+          <t>بيع &lt; تكلفة فعلية؛ بيع &lt; تكلفة محمّلة؛ بيع &lt; تكلفة معيارية؛ هامش دون المستهدف</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>كفته 350 جم ابو هاشم</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>0.06875928741585083</v>
+      </c>
+      <c r="F27" s="44" t="inlineStr">
         <is>
           <t>هامش دون المستهدف</t>
         </is>

</xml_diff>